<commit_message>
chore: Update Testing Set Questions to be self-referential
</commit_message>
<xml_diff>
--- a/Testing Set/Testing Set Questions.xlsx
+++ b/Testing Set/Testing Set Questions.xlsx
@@ -112,16 +112,16 @@
     <t>Testing Set Questions.xlsx</t>
   </si>
   <si>
-    <t>Which question has reference to KFIN’s revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> The question is “What was KFIN's revenue in 2021?”</t>
+    <t>Which question has an answer as ₹4586550000</t>
+  </si>
+  <si>
+    <t>The question is “What was KFIN's revenue in 2021?”</t>
   </si>
   <si>
     <t>Does any question has reference to document 4. C-2015-07-288.pdf, p12</t>
   </si>
   <si>
-    <t>The question is “What metrics helped CCI determine if the combination would be anticompetitive?”</t>
+    <t>It's “What metrics helped CCI determine if the combination would be anticompetitive?”</t>
   </si>
 </sst>
 </file>
@@ -207,7 +207,7 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -433,12 +433,12 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -470,10 +470,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Arial"/>
-            <a:ea typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-            <a:sym typeface="Arial"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -712,12 +712,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1021,10 +1021,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Arial"/>
-            <a:ea typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-            <a:sym typeface="Arial"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1383,7 +1383,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" ht="24.65" customHeight="1">
       <c r="A9" t="s" s="4">
         <v>24</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" t="s" s="4">
         <v>27</v>
       </c>
@@ -1409,7 +1409,7 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" ht="24.65" customHeight="1">
       <c r="A11" t="s" s="4">
         <v>29</v>
       </c>

</xml_diff>